<commit_message>
corection in h2 lhv for tables
</commit_message>
<xml_diff>
--- a/Phi_calc.xlsx
+++ b/Phi_calc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tud365-my.sharepoint.com/personal/fmaiorodrigues_tudelft_nl/Documents/Combustion/Assignments/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="11" documentId="8_{B85172A8-837B-44CC-B559-727F8BB139E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E280228-A03C-43ED-82C6-53C84D57A593}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="8_{B85172A8-837B-44CC-B559-727F8BB139E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21AD5F66-46A1-41DE-B911-AC7888D9F12A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{CEFF3C84-A269-430F-B545-0B81AEC1D7B0}"/>
   </bookViews>
@@ -742,7 +742,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="131">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -788,155 +788,23 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="22" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="16" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="17" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="20" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="20" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="21" borderId="16" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="17" xfId="0" quotePrefix="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="22" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="22" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -946,39 +814,17 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="24" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="12" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="23" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -991,9 +837,158 @@
     <xf numFmtId="0" fontId="0" fillId="14" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="13" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="24" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="11" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="19" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1327,6 +1322,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63027C88-9E38-47B1-8238-A6D33BAC1632}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A2:AF29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -1352,23 +1350,23 @@
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="43" t="s">
+      <c r="R3" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="43"/>
-      <c r="T3" s="43"/>
-      <c r="U3" s="43"/>
-      <c r="V3" s="43"/>
-      <c r="W3" s="43"/>
-      <c r="X3" s="43"/>
-      <c r="Y3" s="43"/>
-      <c r="Z3" s="43"/>
-      <c r="AA3" s="43"/>
-      <c r="AB3" s="43"/>
-      <c r="AC3" s="43"/>
-      <c r="AD3" s="43"/>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="44"/>
+      <c r="S3" s="99"/>
+      <c r="T3" s="99"/>
+      <c r="U3" s="99"/>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99"/>
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="99"/>
+      <c r="AD3" s="99"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="100"/>
     </row>
     <row r="4" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>
@@ -1386,72 +1384,72 @@
       <c r="AF4" s="5"/>
     </row>
     <row r="5" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="47"/>
-      <c r="H5" s="48" t="s">
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="103"/>
+      <c r="H5" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="I5" s="49"/>
-      <c r="J5" s="50"/>
-      <c r="L5" s="66" t="s">
+      <c r="I5" s="95"/>
+      <c r="J5" s="96"/>
+      <c r="L5" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="67"/>
-      <c r="N5" s="68"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="106"/>
       <c r="O5" s="5"/>
       <c r="P5" s="6" t="s">
         <v>2</v>
       </c>
       <c r="Q5" s="4"/>
-      <c r="R5" s="51" t="s">
+      <c r="R5" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="S5" s="52"/>
-      <c r="T5" s="52"/>
-      <c r="U5" s="52"/>
-      <c r="V5" s="53"/>
-      <c r="X5" s="48" t="s">
+      <c r="S5" s="108"/>
+      <c r="T5" s="108"/>
+      <c r="U5" s="108"/>
+      <c r="V5" s="109"/>
+      <c r="X5" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="Y5" s="49"/>
-      <c r="Z5" s="50"/>
-      <c r="AB5" s="82" t="s">
+      <c r="Y5" s="95"/>
+      <c r="Z5" s="96"/>
+      <c r="AB5" s="110" t="s">
         <v>6</v>
       </c>
-      <c r="AC5" s="83"/>
-      <c r="AD5" s="83"/>
-      <c r="AE5" s="83"/>
-      <c r="AF5" s="84"/>
+      <c r="AC5" s="111"/>
+      <c r="AD5" s="111"/>
+      <c r="AE5" s="111"/>
+      <c r="AF5" s="112"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="56"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="86"/>
       <c r="H6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="57" t="s">
+      <c r="I6" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="58"/>
-      <c r="L6" s="85" t="s">
+      <c r="J6" s="98"/>
+      <c r="L6" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="62" t="s">
+      <c r="M6" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="N6" s="63"/>
+      <c r="N6" s="88"/>
       <c r="O6" s="5"/>
       <c r="P6" s="6" t="s">
         <v>2</v>
@@ -1460,28 +1458,28 @@
       <c r="R6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="S6" s="59" t="s">
+      <c r="S6" s="89" t="s">
         <v>11</v>
       </c>
-      <c r="T6" s="60"/>
-      <c r="U6" s="60"/>
-      <c r="V6" s="61"/>
+      <c r="T6" s="90"/>
+      <c r="U6" s="90"/>
+      <c r="V6" s="91"/>
       <c r="X6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="Y6" s="57" t="s">
+      <c r="Y6" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="Z6" s="58"/>
-      <c r="AB6" s="91" t="s">
+      <c r="Z6" s="98"/>
+      <c r="AB6" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="AC6" s="87" t="s">
+      <c r="AC6" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="AD6" s="87"/>
-      <c r="AE6" s="87"/>
-      <c r="AF6" s="88"/>
+      <c r="AD6" s="92"/>
+      <c r="AE6" s="92"/>
+      <c r="AF6" s="93"/>
     </row>
     <row r="7" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="10">
@@ -1509,14 +1507,14 @@
       <c r="J7" s="15">
         <v>2</v>
       </c>
-      <c r="L7" s="86">
+      <c r="L7" s="44">
         <f>(V8+AF8) / 2</f>
         <v>2</v>
       </c>
-      <c r="M7" s="64" t="s">
+      <c r="M7" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="65">
+      <c r="N7" s="38">
         <v>2</v>
       </c>
       <c r="O7" s="5"/>
@@ -1550,20 +1548,20 @@
       <c r="Z7" s="15">
         <v>2</v>
       </c>
-      <c r="AB7" s="92">
+      <c r="AB7" s="48">
         <f>F8/AD7</f>
         <v>2</v>
       </c>
-      <c r="AC7" s="89" t="s">
+      <c r="AC7" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="AD7" s="89">
+      <c r="AD7" s="45">
         <v>2</v>
       </c>
-      <c r="AE7" s="89" t="s">
+      <c r="AE7" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="AF7" s="90">
+      <c r="AF7" s="46">
         <v>1</v>
       </c>
     </row>
@@ -1625,191 +1623,191 @@
     </row>
     <row r="9" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A10" s="69" t="s">
+      <c r="A10" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="71"/>
-      <c r="C10" s="72">
+      <c r="B10" s="41"/>
+      <c r="C10" s="113">
         <v>-74.849999999999994</v>
       </c>
-      <c r="D10" s="73"/>
-      <c r="E10" s="73"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="71"/>
-      <c r="H10" s="71"/>
-      <c r="I10" s="72">
+      <c r="D10" s="114"/>
+      <c r="E10" s="114"/>
+      <c r="F10" s="115"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="113">
         <v>0</v>
       </c>
-      <c r="J10" s="74"/>
-      <c r="K10" s="71"/>
-      <c r="L10" s="71"/>
-      <c r="M10" s="72">
+      <c r="J10" s="115"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="113">
         <v>0</v>
       </c>
-      <c r="N10" s="74"/>
-      <c r="O10" s="71"/>
-      <c r="P10" s="71" t="s">
+      <c r="N10" s="115"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="Q10" s="71"/>
-      <c r="R10" s="71"/>
-      <c r="S10" s="72">
+      <c r="Q10" s="41"/>
+      <c r="R10" s="41"/>
+      <c r="S10" s="113">
         <v>-393</v>
       </c>
-      <c r="T10" s="73"/>
-      <c r="U10" s="73"/>
-      <c r="V10" s="74"/>
-      <c r="W10" s="71"/>
-      <c r="X10" s="71"/>
-      <c r="Y10" s="72">
+      <c r="T10" s="114"/>
+      <c r="U10" s="114"/>
+      <c r="V10" s="115"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="113">
         <v>0</v>
       </c>
-      <c r="Z10" s="74"/>
-      <c r="AA10" s="71"/>
-      <c r="AB10" s="71"/>
-      <c r="AC10" s="72">
+      <c r="Z10" s="115"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="113">
         <v>-241.81</v>
       </c>
-      <c r="AD10" s="73"/>
-      <c r="AE10" s="73"/>
-      <c r="AF10" s="74"/>
+      <c r="AD10" s="114"/>
+      <c r="AE10" s="114"/>
+      <c r="AF10" s="115"/>
     </row>
     <row r="11" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="71"/>
-      <c r="C11" s="75">
+      <c r="B11" s="41"/>
+      <c r="C11" s="116">
         <f>C10*B7</f>
         <v>-74.849999999999994</v>
       </c>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="77"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="71"/>
-      <c r="I11" s="75">
+      <c r="D11" s="117"/>
+      <c r="E11" s="117"/>
+      <c r="F11" s="118"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="116">
         <v>0</v>
       </c>
-      <c r="J11" s="77"/>
-      <c r="K11" s="71"/>
-      <c r="L11" s="71"/>
-      <c r="M11" s="75">
+      <c r="J11" s="118"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="116">
         <f>L7*M10</f>
         <v>0</v>
       </c>
-      <c r="N11" s="77"/>
-      <c r="O11" s="71"/>
-      <c r="P11" s="71" t="s">
+      <c r="N11" s="118"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="Q11" s="71"/>
-      <c r="R11" s="71"/>
-      <c r="S11" s="75">
+      <c r="Q11" s="41"/>
+      <c r="R11" s="41"/>
+      <c r="S11" s="116">
         <f>S10*R7</f>
         <v>-393</v>
       </c>
-      <c r="T11" s="76"/>
-      <c r="U11" s="76"/>
-      <c r="V11" s="77"/>
-      <c r="W11" s="78"/>
-      <c r="X11" s="78"/>
-      <c r="Y11" s="75">
+      <c r="T11" s="117"/>
+      <c r="U11" s="117"/>
+      <c r="V11" s="118"/>
+      <c r="W11" s="42"/>
+      <c r="X11" s="42"/>
+      <c r="Y11" s="116">
         <v>0</v>
       </c>
-      <c r="Z11" s="77"/>
-      <c r="AA11" s="78"/>
-      <c r="AB11" s="78"/>
-      <c r="AC11" s="75">
+      <c r="Z11" s="118"/>
+      <c r="AA11" s="42"/>
+      <c r="AB11" s="42"/>
+      <c r="AC11" s="116">
         <f>AC10*AB7</f>
         <v>-483.62</v>
       </c>
-      <c r="AD11" s="76"/>
-      <c r="AE11" s="76"/>
-      <c r="AF11" s="77"/>
+      <c r="AD11" s="117"/>
+      <c r="AE11" s="117"/>
+      <c r="AF11" s="118"/>
     </row>
     <row r="12" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="13" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="70" t="s">
+      <c r="A13" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="79">
+      <c r="B13" s="120">
         <f>C11+M11</f>
         <v>-74.849999999999994</v>
       </c>
-      <c r="C13" s="80"/>
-      <c r="D13" s="80"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="80"/>
-      <c r="G13" s="80"/>
-      <c r="H13" s="80"/>
-      <c r="I13" s="80"/>
-      <c r="J13" s="80"/>
-      <c r="K13" s="80"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="80"/>
-      <c r="N13" s="80"/>
-      <c r="O13" s="81"/>
-      <c r="P13" s="71"/>
-      <c r="Q13" s="79">
+      <c r="C13" s="121"/>
+      <c r="D13" s="121"/>
+      <c r="E13" s="121"/>
+      <c r="F13" s="121"/>
+      <c r="G13" s="121"/>
+      <c r="H13" s="121"/>
+      <c r="I13" s="121"/>
+      <c r="J13" s="121"/>
+      <c r="K13" s="121"/>
+      <c r="L13" s="121"/>
+      <c r="M13" s="121"/>
+      <c r="N13" s="121"/>
+      <c r="O13" s="122"/>
+      <c r="P13" s="41"/>
+      <c r="Q13" s="120">
         <f>S11+AC11</f>
         <v>-876.62</v>
       </c>
-      <c r="R13" s="80"/>
-      <c r="S13" s="80"/>
-      <c r="T13" s="80"/>
-      <c r="U13" s="80"/>
-      <c r="V13" s="80"/>
-      <c r="W13" s="80"/>
-      <c r="X13" s="80"/>
-      <c r="Y13" s="80"/>
-      <c r="Z13" s="80"/>
-      <c r="AA13" s="80"/>
-      <c r="AB13" s="80"/>
-      <c r="AC13" s="80"/>
-      <c r="AD13" s="80"/>
-      <c r="AE13" s="80"/>
-      <c r="AF13" s="81"/>
+      <c r="R13" s="121"/>
+      <c r="S13" s="121"/>
+      <c r="T13" s="121"/>
+      <c r="U13" s="121"/>
+      <c r="V13" s="121"/>
+      <c r="W13" s="121"/>
+      <c r="X13" s="121"/>
+      <c r="Y13" s="121"/>
+      <c r="Z13" s="121"/>
+      <c r="AA13" s="121"/>
+      <c r="AB13" s="121"/>
+      <c r="AC13" s="121"/>
+      <c r="AD13" s="121"/>
+      <c r="AE13" s="121"/>
+      <c r="AF13" s="122"/>
     </row>
     <row r="14" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="15" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="70" t="s">
+      <c r="A15" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="79">
+      <c r="B15" s="120">
         <f>Q13-B13</f>
         <v>-801.77</v>
       </c>
-      <c r="C15" s="80"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="80"/>
-      <c r="G15" s="80"/>
-      <c r="H15" s="80"/>
-      <c r="I15" s="80"/>
-      <c r="J15" s="80"/>
-      <c r="K15" s="80"/>
-      <c r="L15" s="80"/>
-      <c r="M15" s="80"/>
-      <c r="N15" s="80"/>
-      <c r="O15" s="80"/>
-      <c r="P15" s="80"/>
-      <c r="Q15" s="80"/>
-      <c r="R15" s="80"/>
-      <c r="S15" s="80"/>
-      <c r="T15" s="80"/>
-      <c r="U15" s="80"/>
-      <c r="V15" s="80"/>
-      <c r="W15" s="80"/>
-      <c r="X15" s="80"/>
-      <c r="Y15" s="80"/>
-      <c r="Z15" s="80"/>
-      <c r="AA15" s="80"/>
-      <c r="AB15" s="80"/>
-      <c r="AC15" s="80"/>
-      <c r="AD15" s="80"/>
-      <c r="AE15" s="80"/>
-      <c r="AF15" s="81"/>
+      <c r="C15" s="121"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="121"/>
+      <c r="F15" s="121"/>
+      <c r="G15" s="121"/>
+      <c r="H15" s="121"/>
+      <c r="I15" s="121"/>
+      <c r="J15" s="121"/>
+      <c r="K15" s="121"/>
+      <c r="L15" s="121"/>
+      <c r="M15" s="121"/>
+      <c r="N15" s="121"/>
+      <c r="O15" s="121"/>
+      <c r="P15" s="121"/>
+      <c r="Q15" s="121"/>
+      <c r="R15" s="121"/>
+      <c r="S15" s="121"/>
+      <c r="T15" s="121"/>
+      <c r="U15" s="121"/>
+      <c r="V15" s="121"/>
+      <c r="W15" s="121"/>
+      <c r="X15" s="121"/>
+      <c r="Y15" s="121"/>
+      <c r="Z15" s="121"/>
+      <c r="AA15" s="121"/>
+      <c r="AB15" s="121"/>
+      <c r="AC15" s="121"/>
+      <c r="AD15" s="121"/>
+      <c r="AE15" s="121"/>
+      <c r="AF15" s="122"/>
     </row>
     <row r="17" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -1817,27 +1815,27 @@
         <v>21</v>
       </c>
       <c r="B18" s="26"/>
-      <c r="C18" s="40">
+      <c r="C18" s="123">
         <f>D7*C21+F7*F21</f>
         <v>16.032</v>
       </c>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="42"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
+      <c r="F18" s="125"/>
       <c r="G18" s="26"/>
       <c r="H18" s="26"/>
-      <c r="I18" s="40">
+      <c r="I18" s="123">
         <f>J7*J21</f>
         <v>28</v>
       </c>
-      <c r="J18" s="42"/>
+      <c r="J18" s="125"/>
       <c r="K18" s="26"/>
       <c r="L18" s="26"/>
-      <c r="M18" s="40">
+      <c r="M18" s="123">
         <f>N7*M21</f>
         <v>32</v>
       </c>
-      <c r="N18" s="42"/>
+      <c r="N18" s="125"/>
       <c r="O18" s="27" t="s">
         <v>22</v>
       </c>
@@ -1846,56 +1844,56 @@
         <v>22</v>
       </c>
       <c r="R18" s="26"/>
-      <c r="S18" s="40">
+      <c r="S18" s="123">
         <f>T7*C21+V7*M21</f>
         <v>44</v>
       </c>
-      <c r="T18" s="41"/>
-      <c r="U18" s="41"/>
-      <c r="V18" s="42"/>
+      <c r="T18" s="124"/>
+      <c r="U18" s="124"/>
+      <c r="V18" s="125"/>
       <c r="W18" s="26"/>
       <c r="X18" s="26"/>
-      <c r="Y18" s="40">
+      <c r="Y18" s="123">
         <f>J21*Z7</f>
         <v>28</v>
       </c>
-      <c r="Z18" s="42"/>
+      <c r="Z18" s="125"/>
       <c r="AA18" s="26"/>
       <c r="AB18" s="26"/>
-      <c r="AC18" s="40">
+      <c r="AC18" s="123">
         <f>AD7*F21+AF7*M21</f>
         <v>18.015999999999998</v>
       </c>
-      <c r="AD18" s="41"/>
-      <c r="AE18" s="41"/>
-      <c r="AF18" s="42"/>
+      <c r="AD18" s="124"/>
+      <c r="AE18" s="124"/>
+      <c r="AF18" s="125"/>
     </row>
     <row r="19" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="28" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="26"/>
-      <c r="C19" s="37">
+      <c r="C19" s="82">
         <f>C18*B7</f>
         <v>16.032</v>
       </c>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
+      <c r="D19" s="119"/>
+      <c r="E19" s="119"/>
+      <c r="F19" s="83"/>
       <c r="G19" s="26"/>
       <c r="H19" s="26"/>
-      <c r="I19" s="37">
+      <c r="I19" s="82">
         <f>I18*H7</f>
         <v>208.32000000000002</v>
       </c>
-      <c r="J19" s="39"/>
+      <c r="J19" s="83"/>
       <c r="K19" s="26"/>
       <c r="L19" s="26"/>
-      <c r="M19" s="37">
+      <c r="M19" s="82">
         <f>M18*L7</f>
         <v>64</v>
       </c>
-      <c r="N19" s="39"/>
+      <c r="N19" s="83"/>
       <c r="O19" s="29">
         <f>M19+C19+I19</f>
         <v>288.35200000000003</v>
@@ -1906,35 +1904,35 @@
         <v>288.35200000000003</v>
       </c>
       <c r="R19" s="26"/>
-      <c r="S19" s="37">
+      <c r="S19" s="82">
         <f>S18*R7</f>
         <v>44</v>
       </c>
-      <c r="T19" s="38"/>
-      <c r="U19" s="38">
+      <c r="T19" s="119"/>
+      <c r="U19" s="119">
         <f t="shared" ref="U19" si="0">U18*T7</f>
         <v>0</v>
       </c>
-      <c r="V19" s="39"/>
+      <c r="V19" s="83"/>
       <c r="W19" s="26"/>
       <c r="X19" s="26"/>
-      <c r="Y19" s="37">
+      <c r="Y19" s="82">
         <f>Y18*X7</f>
         <v>208.32000000000002</v>
       </c>
-      <c r="Z19" s="39"/>
+      <c r="Z19" s="83"/>
       <c r="AA19" s="26"/>
       <c r="AB19" s="26"/>
-      <c r="AC19" s="37">
+      <c r="AC19" s="82">
         <f>AC18*AB7</f>
         <v>36.031999999999996</v>
       </c>
-      <c r="AD19" s="38"/>
-      <c r="AE19" s="38">
+      <c r="AD19" s="119"/>
+      <c r="AE19" s="119">
         <f t="shared" ref="AE19" si="1">AE18*AD7</f>
         <v>0</v>
       </c>
-      <c r="AF19" s="39"/>
+      <c r="AF19" s="83"/>
     </row>
     <row r="20" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="21" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2034,16 +2032,15 @@
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="Y19:Z19"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="AC6:AF6"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="X5:Z5"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="R3:AF3"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="Y18:Z18"/>
+    <mergeCell ref="Q13:AF13"/>
+    <mergeCell ref="B15:AF15"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="M18:N18"/>
+    <mergeCell ref="S18:V18"/>
+    <mergeCell ref="AC18:AF18"/>
+    <mergeCell ref="I18:J18"/>
     <mergeCell ref="B5:F5"/>
     <mergeCell ref="L5:N5"/>
     <mergeCell ref="R5:V5"/>
@@ -2052,35 +2049,40 @@
     <mergeCell ref="M10:N10"/>
     <mergeCell ref="S10:V10"/>
     <mergeCell ref="AC10:AF10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="Y10:Z10"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="X5:Z5"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="R3:AF3"/>
+    <mergeCell ref="Y19:Z19"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="AC6:AF6"/>
     <mergeCell ref="C11:F11"/>
     <mergeCell ref="M11:N11"/>
     <mergeCell ref="S11:V11"/>
     <mergeCell ref="AC11:AF11"/>
-    <mergeCell ref="I10:J10"/>
     <mergeCell ref="I11:J11"/>
-    <mergeCell ref="Y10:Z10"/>
     <mergeCell ref="Y11:Z11"/>
     <mergeCell ref="C19:F19"/>
     <mergeCell ref="M19:N19"/>
     <mergeCell ref="S19:V19"/>
     <mergeCell ref="AC19:AF19"/>
     <mergeCell ref="B13:O13"/>
-    <mergeCell ref="Q13:AF13"/>
-    <mergeCell ref="B15:AF15"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="M18:N18"/>
-    <mergeCell ref="S18:V18"/>
-    <mergeCell ref="AC18:AF18"/>
-    <mergeCell ref="I18:J18"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="Y18:Z18"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42775804-EF79-4D2A-9A15-37A9953A5ACE}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A2:AF29"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2106,23 +2108,23 @@
       <c r="N3" s="2"/>
       <c r="O3" s="3"/>
       <c r="Q3" s="1"/>
-      <c r="R3" s="43" t="s">
+      <c r="R3" s="99" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="43"/>
-      <c r="T3" s="43"/>
-      <c r="U3" s="43"/>
-      <c r="V3" s="43"/>
-      <c r="W3" s="43"/>
-      <c r="X3" s="43"/>
-      <c r="Y3" s="43"/>
-      <c r="Z3" s="43"/>
-      <c r="AA3" s="43"/>
-      <c r="AB3" s="43"/>
-      <c r="AC3" s="43"/>
-      <c r="AD3" s="43"/>
-      <c r="AE3" s="43"/>
-      <c r="AF3" s="44"/>
+      <c r="S3" s="99"/>
+      <c r="T3" s="99"/>
+      <c r="U3" s="99"/>
+      <c r="V3" s="99"/>
+      <c r="W3" s="99"/>
+      <c r="X3" s="99"/>
+      <c r="Y3" s="99"/>
+      <c r="Z3" s="99"/>
+      <c r="AA3" s="99"/>
+      <c r="AB3" s="99"/>
+      <c r="AC3" s="99"/>
+      <c r="AD3" s="99"/>
+      <c r="AE3" s="99"/>
+      <c r="AF3" s="100"/>
     </row>
     <row r="4" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B4" s="4"/>
@@ -2140,72 +2142,72 @@
       <c r="AF4" s="5"/>
     </row>
     <row r="5" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="45" t="s">
+      <c r="B5" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="46"/>
-      <c r="D5" s="46"/>
-      <c r="E5" s="46"/>
-      <c r="F5" s="47"/>
-      <c r="H5" s="48" t="s">
+      <c r="C5" s="102"/>
+      <c r="D5" s="102"/>
+      <c r="E5" s="102"/>
+      <c r="F5" s="103"/>
+      <c r="H5" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="I5" s="49"/>
-      <c r="J5" s="50"/>
-      <c r="L5" s="66" t="s">
+      <c r="I5" s="95"/>
+      <c r="J5" s="96"/>
+      <c r="L5" s="104" t="s">
         <v>4</v>
       </c>
-      <c r="M5" s="67"/>
-      <c r="N5" s="68"/>
+      <c r="M5" s="105"/>
+      <c r="N5" s="106"/>
       <c r="O5" s="5"/>
       <c r="P5" s="6" t="s">
         <v>2</v>
       </c>
       <c r="Q5" s="4"/>
-      <c r="R5" s="51" t="s">
+      <c r="R5" s="107" t="s">
         <v>5</v>
       </c>
-      <c r="S5" s="52"/>
-      <c r="T5" s="52"/>
-      <c r="U5" s="52"/>
-      <c r="V5" s="53"/>
-      <c r="X5" s="48" t="s">
+      <c r="S5" s="108"/>
+      <c r="T5" s="108"/>
+      <c r="U5" s="108"/>
+      <c r="V5" s="109"/>
+      <c r="X5" s="94" t="s">
         <v>28</v>
       </c>
-      <c r="Y5" s="49"/>
-      <c r="Z5" s="50"/>
-      <c r="AB5" s="82" t="s">
+      <c r="Y5" s="95"/>
+      <c r="Z5" s="96"/>
+      <c r="AB5" s="110" t="s">
         <v>6</v>
       </c>
-      <c r="AC5" s="83"/>
-      <c r="AD5" s="83"/>
-      <c r="AE5" s="83"/>
-      <c r="AF5" s="84"/>
+      <c r="AC5" s="111"/>
+      <c r="AD5" s="111"/>
+      <c r="AE5" s="111"/>
+      <c r="AF5" s="112"/>
     </row>
     <row r="6" spans="1:32" x14ac:dyDescent="0.3">
       <c r="B6" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="54" t="s">
+      <c r="C6" s="84" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="55"/>
-      <c r="E6" s="55"/>
-      <c r="F6" s="56"/>
+      <c r="D6" s="85"/>
+      <c r="E6" s="85"/>
+      <c r="F6" s="86"/>
       <c r="H6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="I6" s="57" t="s">
+      <c r="I6" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="J6" s="58"/>
-      <c r="L6" s="85" t="s">
+      <c r="J6" s="98"/>
+      <c r="L6" s="43" t="s">
         <v>9</v>
       </c>
-      <c r="M6" s="62" t="s">
+      <c r="M6" s="87" t="s">
         <v>10</v>
       </c>
-      <c r="N6" s="63"/>
+      <c r="N6" s="88"/>
       <c r="O6" s="5"/>
       <c r="P6" s="6" t="s">
         <v>2</v>
@@ -2214,28 +2216,28 @@
       <c r="R6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="S6" s="59" t="s">
+      <c r="S6" s="89" t="s">
         <v>11</v>
       </c>
-      <c r="T6" s="60"/>
-      <c r="U6" s="60"/>
-      <c r="V6" s="61"/>
+      <c r="T6" s="90"/>
+      <c r="U6" s="90"/>
+      <c r="V6" s="91"/>
       <c r="X6" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="Y6" s="57" t="s">
+      <c r="Y6" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="Z6" s="58"/>
-      <c r="AB6" s="91" t="s">
+      <c r="Z6" s="98"/>
+      <c r="AB6" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="AC6" s="87" t="s">
+      <c r="AC6" s="92" t="s">
         <v>11</v>
       </c>
-      <c r="AD6" s="87"/>
-      <c r="AE6" s="87"/>
-      <c r="AF6" s="88"/>
+      <c r="AD6" s="92"/>
+      <c r="AE6" s="92"/>
+      <c r="AF6" s="93"/>
     </row>
     <row r="7" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B7" s="10">
@@ -2244,7 +2246,7 @@
       <c r="C7" s="11" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="94">
+      <c r="D7" s="50">
         <v>0</v>
       </c>
       <c r="E7" s="11" t="s">
@@ -2263,14 +2265,14 @@
       <c r="J7" s="15">
         <v>2</v>
       </c>
-      <c r="L7" s="86">
+      <c r="L7" s="44">
         <f>(V8+AF8) / 2</f>
         <v>0.5</v>
       </c>
-      <c r="M7" s="64" t="s">
+      <c r="M7" s="37" t="s">
         <v>15</v>
       </c>
-      <c r="N7" s="65">
+      <c r="N7" s="38">
         <v>2</v>
       </c>
       <c r="O7" s="5"/>
@@ -2304,20 +2306,20 @@
       <c r="Z7" s="15">
         <v>2</v>
       </c>
-      <c r="AB7" s="92">
+      <c r="AB7" s="48">
         <f>F8/AD7</f>
         <v>1</v>
       </c>
-      <c r="AC7" s="89" t="s">
+      <c r="AC7" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="AD7" s="89">
+      <c r="AD7" s="45">
         <v>2</v>
       </c>
-      <c r="AE7" s="89" t="s">
+      <c r="AE7" s="45" t="s">
         <v>15</v>
       </c>
-      <c r="AF7" s="90">
+      <c r="AF7" s="46">
         <v>1</v>
       </c>
     </row>
@@ -2379,191 +2381,191 @@
     </row>
     <row r="9" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="10" spans="1:32" x14ac:dyDescent="0.3">
-      <c r="A10" s="69" t="s">
+      <c r="A10" s="39" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="71"/>
-      <c r="C10" s="72">
+      <c r="B10" s="41"/>
+      <c r="C10" s="113">
         <v>0</v>
       </c>
-      <c r="D10" s="73"/>
-      <c r="E10" s="73"/>
-      <c r="F10" s="74"/>
-      <c r="G10" s="71"/>
-      <c r="H10" s="71"/>
-      <c r="I10" s="72">
+      <c r="D10" s="114"/>
+      <c r="E10" s="114"/>
+      <c r="F10" s="115"/>
+      <c r="G10" s="41"/>
+      <c r="H10" s="41"/>
+      <c r="I10" s="113">
         <v>0</v>
       </c>
-      <c r="J10" s="74"/>
-      <c r="K10" s="71"/>
-      <c r="L10" s="71"/>
-      <c r="M10" s="72">
+      <c r="J10" s="115"/>
+      <c r="K10" s="41"/>
+      <c r="L10" s="41"/>
+      <c r="M10" s="113">
         <v>0</v>
       </c>
-      <c r="N10" s="74"/>
-      <c r="O10" s="71"/>
-      <c r="P10" s="71" t="s">
+      <c r="N10" s="115"/>
+      <c r="O10" s="41"/>
+      <c r="P10" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="Q10" s="71"/>
-      <c r="R10" s="71"/>
-      <c r="S10" s="72">
+      <c r="Q10" s="41"/>
+      <c r="R10" s="41"/>
+      <c r="S10" s="113">
         <v>-393</v>
       </c>
-      <c r="T10" s="73"/>
-      <c r="U10" s="73"/>
-      <c r="V10" s="74"/>
-      <c r="W10" s="71"/>
-      <c r="X10" s="71"/>
-      <c r="Y10" s="72">
+      <c r="T10" s="114"/>
+      <c r="U10" s="114"/>
+      <c r="V10" s="115"/>
+      <c r="W10" s="41"/>
+      <c r="X10" s="41"/>
+      <c r="Y10" s="113">
         <v>0</v>
       </c>
-      <c r="Z10" s="74"/>
-      <c r="AA10" s="71"/>
-      <c r="AB10" s="71"/>
-      <c r="AC10" s="72">
+      <c r="Z10" s="115"/>
+      <c r="AA10" s="41"/>
+      <c r="AB10" s="41"/>
+      <c r="AC10" s="113">
         <v>-241.81</v>
       </c>
-      <c r="AD10" s="73"/>
-      <c r="AE10" s="73"/>
-      <c r="AF10" s="74"/>
+      <c r="AD10" s="114"/>
+      <c r="AE10" s="114"/>
+      <c r="AF10" s="115"/>
     </row>
     <row r="11" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A11" s="70" t="s">
+      <c r="A11" s="40" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="71"/>
-      <c r="C11" s="75">
+      <c r="B11" s="41"/>
+      <c r="C11" s="116">
         <f>C10*B7</f>
         <v>0</v>
       </c>
-      <c r="D11" s="76"/>
-      <c r="E11" s="76"/>
-      <c r="F11" s="77"/>
-      <c r="G11" s="71"/>
-      <c r="H11" s="71"/>
-      <c r="I11" s="75">
+      <c r="D11" s="117"/>
+      <c r="E11" s="117"/>
+      <c r="F11" s="118"/>
+      <c r="G11" s="41"/>
+      <c r="H11" s="41"/>
+      <c r="I11" s="116">
         <v>0</v>
       </c>
-      <c r="J11" s="77"/>
-      <c r="K11" s="71"/>
-      <c r="L11" s="71"/>
-      <c r="M11" s="75">
+      <c r="J11" s="118"/>
+      <c r="K11" s="41"/>
+      <c r="L11" s="41"/>
+      <c r="M11" s="116">
         <f>L7*M10</f>
         <v>0</v>
       </c>
-      <c r="N11" s="77"/>
-      <c r="O11" s="71"/>
-      <c r="P11" s="71" t="s">
+      <c r="N11" s="118"/>
+      <c r="O11" s="41"/>
+      <c r="P11" s="41" t="s">
         <v>2</v>
       </c>
-      <c r="Q11" s="71"/>
-      <c r="R11" s="71"/>
-      <c r="S11" s="75">
+      <c r="Q11" s="41"/>
+      <c r="R11" s="41"/>
+      <c r="S11" s="116">
         <f>S10*R7</f>
         <v>0</v>
       </c>
-      <c r="T11" s="76"/>
-      <c r="U11" s="76"/>
-      <c r="V11" s="77"/>
-      <c r="W11" s="78"/>
-      <c r="X11" s="78"/>
-      <c r="Y11" s="75">
+      <c r="T11" s="117"/>
+      <c r="U11" s="117"/>
+      <c r="V11" s="118"/>
+      <c r="W11" s="42"/>
+      <c r="X11" s="42"/>
+      <c r="Y11" s="116">
         <v>0</v>
       </c>
-      <c r="Z11" s="77"/>
-      <c r="AA11" s="78"/>
-      <c r="AB11" s="78"/>
-      <c r="AC11" s="75">
+      <c r="Z11" s="118"/>
+      <c r="AA11" s="42"/>
+      <c r="AB11" s="42"/>
+      <c r="AC11" s="116">
         <f>AC10*AB7</f>
         <v>-241.81</v>
       </c>
-      <c r="AD11" s="76"/>
-      <c r="AE11" s="76"/>
-      <c r="AF11" s="77"/>
+      <c r="AD11" s="117"/>
+      <c r="AE11" s="117"/>
+      <c r="AF11" s="118"/>
     </row>
     <row r="12" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="13" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="70" t="s">
+      <c r="A13" s="40" t="s">
         <v>19</v>
       </c>
-      <c r="B13" s="79">
+      <c r="B13" s="120">
         <f>C11+M11</f>
         <v>0</v>
       </c>
-      <c r="C13" s="80"/>
-      <c r="D13" s="80"/>
-      <c r="E13" s="80"/>
-      <c r="F13" s="80"/>
-      <c r="G13" s="80"/>
-      <c r="H13" s="80"/>
-      <c r="I13" s="80"/>
-      <c r="J13" s="80"/>
-      <c r="K13" s="80"/>
-      <c r="L13" s="80"/>
-      <c r="M13" s="80"/>
-      <c r="N13" s="80"/>
-      <c r="O13" s="81"/>
-      <c r="P13" s="71"/>
-      <c r="Q13" s="79">
+      <c r="C13" s="121"/>
+      <c r="D13" s="121"/>
+      <c r="E13" s="121"/>
+      <c r="F13" s="121"/>
+      <c r="G13" s="121"/>
+      <c r="H13" s="121"/>
+      <c r="I13" s="121"/>
+      <c r="J13" s="121"/>
+      <c r="K13" s="121"/>
+      <c r="L13" s="121"/>
+      <c r="M13" s="121"/>
+      <c r="N13" s="121"/>
+      <c r="O13" s="122"/>
+      <c r="P13" s="41"/>
+      <c r="Q13" s="120">
         <f>S11+AC11</f>
         <v>-241.81</v>
       </c>
-      <c r="R13" s="80"/>
-      <c r="S13" s="80"/>
-      <c r="T13" s="80"/>
-      <c r="U13" s="80"/>
-      <c r="V13" s="80"/>
-      <c r="W13" s="80"/>
-      <c r="X13" s="80"/>
-      <c r="Y13" s="80"/>
-      <c r="Z13" s="80"/>
-      <c r="AA13" s="80"/>
-      <c r="AB13" s="80"/>
-      <c r="AC13" s="80"/>
-      <c r="AD13" s="80"/>
-      <c r="AE13" s="80"/>
-      <c r="AF13" s="81"/>
+      <c r="R13" s="121"/>
+      <c r="S13" s="121"/>
+      <c r="T13" s="121"/>
+      <c r="U13" s="121"/>
+      <c r="V13" s="121"/>
+      <c r="W13" s="121"/>
+      <c r="X13" s="121"/>
+      <c r="Y13" s="121"/>
+      <c r="Z13" s="121"/>
+      <c r="AA13" s="121"/>
+      <c r="AB13" s="121"/>
+      <c r="AC13" s="121"/>
+      <c r="AD13" s="121"/>
+      <c r="AE13" s="121"/>
+      <c r="AF13" s="122"/>
     </row>
     <row r="14" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="15" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A15" s="70" t="s">
+      <c r="A15" s="40" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="79">
+      <c r="B15" s="120">
         <f>Q13-B13</f>
         <v>-241.81</v>
       </c>
-      <c r="C15" s="80"/>
-      <c r="D15" s="80"/>
-      <c r="E15" s="80"/>
-      <c r="F15" s="80"/>
-      <c r="G15" s="80"/>
-      <c r="H15" s="80"/>
-      <c r="I15" s="80"/>
-      <c r="J15" s="80"/>
-      <c r="K15" s="80"/>
-      <c r="L15" s="80"/>
-      <c r="M15" s="80"/>
-      <c r="N15" s="80"/>
-      <c r="O15" s="80"/>
-      <c r="P15" s="80"/>
-      <c r="Q15" s="80"/>
-      <c r="R15" s="80"/>
-      <c r="S15" s="80"/>
-      <c r="T15" s="80"/>
-      <c r="U15" s="80"/>
-      <c r="V15" s="80"/>
-      <c r="W15" s="80"/>
-      <c r="X15" s="80"/>
-      <c r="Y15" s="80"/>
-      <c r="Z15" s="80"/>
-      <c r="AA15" s="80"/>
-      <c r="AB15" s="80"/>
-      <c r="AC15" s="80"/>
-      <c r="AD15" s="80"/>
-      <c r="AE15" s="80"/>
-      <c r="AF15" s="81"/>
+      <c r="C15" s="121"/>
+      <c r="D15" s="121"/>
+      <c r="E15" s="121"/>
+      <c r="F15" s="121"/>
+      <c r="G15" s="121"/>
+      <c r="H15" s="121"/>
+      <c r="I15" s="121"/>
+      <c r="J15" s="121"/>
+      <c r="K15" s="121"/>
+      <c r="L15" s="121"/>
+      <c r="M15" s="121"/>
+      <c r="N15" s="121"/>
+      <c r="O15" s="121"/>
+      <c r="P15" s="121"/>
+      <c r="Q15" s="121"/>
+      <c r="R15" s="121"/>
+      <c r="S15" s="121"/>
+      <c r="T15" s="121"/>
+      <c r="U15" s="121"/>
+      <c r="V15" s="121"/>
+      <c r="W15" s="121"/>
+      <c r="X15" s="121"/>
+      <c r="Y15" s="121"/>
+      <c r="Z15" s="121"/>
+      <c r="AA15" s="121"/>
+      <c r="AB15" s="121"/>
+      <c r="AC15" s="121"/>
+      <c r="AD15" s="121"/>
+      <c r="AE15" s="121"/>
+      <c r="AF15" s="122"/>
     </row>
     <row r="17" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="18" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2571,27 +2573,27 @@
         <v>21</v>
       </c>
       <c r="B18" s="26"/>
-      <c r="C18" s="40">
+      <c r="C18" s="123">
         <f>D7*C21+F7*F21</f>
         <v>2.016</v>
       </c>
-      <c r="D18" s="41"/>
-      <c r="E18" s="41"/>
-      <c r="F18" s="42"/>
+      <c r="D18" s="124"/>
+      <c r="E18" s="124"/>
+      <c r="F18" s="125"/>
       <c r="G18" s="26"/>
       <c r="H18" s="26"/>
-      <c r="I18" s="40">
+      <c r="I18" s="123">
         <f>J7*J21</f>
         <v>28</v>
       </c>
-      <c r="J18" s="42"/>
+      <c r="J18" s="125"/>
       <c r="K18" s="26"/>
       <c r="L18" s="26"/>
-      <c r="M18" s="40">
+      <c r="M18" s="123">
         <f>N7*M21</f>
         <v>32</v>
       </c>
-      <c r="N18" s="42"/>
+      <c r="N18" s="125"/>
       <c r="O18" s="27" t="s">
         <v>22</v>
       </c>
@@ -2600,56 +2602,56 @@
         <v>22</v>
       </c>
       <c r="R18" s="26"/>
-      <c r="S18" s="40">
+      <c r="S18" s="123">
         <f>T7*C21+V7*M21</f>
         <v>44</v>
       </c>
-      <c r="T18" s="41"/>
-      <c r="U18" s="41"/>
-      <c r="V18" s="42"/>
+      <c r="T18" s="124"/>
+      <c r="U18" s="124"/>
+      <c r="V18" s="125"/>
       <c r="W18" s="26"/>
       <c r="X18" s="26"/>
-      <c r="Y18" s="40">
+      <c r="Y18" s="123">
         <f>J21*Z7</f>
         <v>28</v>
       </c>
-      <c r="Z18" s="42"/>
+      <c r="Z18" s="125"/>
       <c r="AA18" s="26"/>
       <c r="AB18" s="26"/>
-      <c r="AC18" s="40">
+      <c r="AC18" s="123">
         <f>AD7*F21+AF7*M21</f>
         <v>18.015999999999998</v>
       </c>
-      <c r="AD18" s="41"/>
-      <c r="AE18" s="41"/>
-      <c r="AF18" s="42"/>
+      <c r="AD18" s="124"/>
+      <c r="AE18" s="124"/>
+      <c r="AF18" s="125"/>
     </row>
     <row r="19" spans="1:32" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A19" s="28" t="s">
         <v>23</v>
       </c>
       <c r="B19" s="26"/>
-      <c r="C19" s="37">
+      <c r="C19" s="82">
         <f>C18*B7</f>
         <v>2.016</v>
       </c>
-      <c r="D19" s="38"/>
-      <c r="E19" s="38"/>
-      <c r="F19" s="39"/>
+      <c r="D19" s="119"/>
+      <c r="E19" s="119"/>
+      <c r="F19" s="83"/>
       <c r="G19" s="26"/>
       <c r="H19" s="26"/>
-      <c r="I19" s="37">
+      <c r="I19" s="82">
         <f>I18*H7</f>
         <v>52.080000000000005</v>
       </c>
-      <c r="J19" s="39"/>
+      <c r="J19" s="83"/>
       <c r="K19" s="26"/>
       <c r="L19" s="26"/>
-      <c r="M19" s="37">
+      <c r="M19" s="82">
         <f>M18*L7</f>
         <v>16</v>
       </c>
-      <c r="N19" s="39"/>
+      <c r="N19" s="83"/>
       <c r="O19" s="29">
         <f>M19+C19+I19</f>
         <v>70.096000000000004</v>
@@ -2660,35 +2662,35 @@
         <v>70.096000000000004</v>
       </c>
       <c r="R19" s="26"/>
-      <c r="S19" s="37">
+      <c r="S19" s="82">
         <f>S18*R7</f>
         <v>0</v>
       </c>
-      <c r="T19" s="38"/>
-      <c r="U19" s="38">
+      <c r="T19" s="119"/>
+      <c r="U19" s="119">
         <f t="shared" ref="U19" si="0">U18*T7</f>
         <v>0</v>
       </c>
-      <c r="V19" s="39"/>
+      <c r="V19" s="83"/>
       <c r="W19" s="26"/>
       <c r="X19" s="26"/>
-      <c r="Y19" s="37">
+      <c r="Y19" s="82">
         <f>Y18*X7</f>
         <v>52.080000000000005</v>
       </c>
-      <c r="Z19" s="39"/>
+      <c r="Z19" s="83"/>
       <c r="AA19" s="26"/>
       <c r="AB19" s="26"/>
-      <c r="AC19" s="37">
+      <c r="AC19" s="82">
         <f>AC18*AB7</f>
         <v>18.015999999999998</v>
       </c>
-      <c r="AD19" s="38"/>
-      <c r="AE19" s="38">
+      <c r="AD19" s="119"/>
+      <c r="AE19" s="119">
         <f t="shared" ref="AE19" si="1">AE18*AD7</f>
         <v>0</v>
       </c>
-      <c r="AF19" s="39"/>
+      <c r="AF19" s="83"/>
     </row>
     <row r="20" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="21" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
@@ -2769,30 +2771,50 @@
       </c>
     </row>
     <row r="28" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="95" t="s">
+      <c r="A28" s="51" t="s">
         <v>31</v>
       </c>
-      <c r="B28" s="96">
+      <c r="B28" s="52">
         <f>1/B26</f>
         <v>7.9365079365079367</v>
       </c>
     </row>
     <row r="29" spans="1:32" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="97" t="s">
+      <c r="A29" s="53" t="s">
         <v>32</v>
       </c>
-      <c r="B29" s="98">
+      <c r="B29" s="54">
         <f>1/B27</f>
         <v>33.76984126984128</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="40">
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="I19:J19"/>
-    <mergeCell ref="M19:N19"/>
-    <mergeCell ref="S19:V19"/>
-    <mergeCell ref="Y19:Z19"/>
+    <mergeCell ref="AC6:AF6"/>
+    <mergeCell ref="R3:AF3"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="H5:J5"/>
+    <mergeCell ref="L5:N5"/>
+    <mergeCell ref="R5:V5"/>
+    <mergeCell ref="X5:Z5"/>
+    <mergeCell ref="AB5:AF5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="I6:J6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="S6:V6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AC11:AF11"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="I10:J10"/>
+    <mergeCell ref="M10:N10"/>
+    <mergeCell ref="S10:V10"/>
+    <mergeCell ref="Y10:Z10"/>
+    <mergeCell ref="AC10:AF10"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="M11:N11"/>
+    <mergeCell ref="S11:V11"/>
+    <mergeCell ref="Y11:Z11"/>
     <mergeCell ref="AC19:AF19"/>
     <mergeCell ref="B13:O13"/>
     <mergeCell ref="Q13:AF13"/>
@@ -2803,38 +2825,22 @@
     <mergeCell ref="S18:V18"/>
     <mergeCell ref="Y18:Z18"/>
     <mergeCell ref="AC18:AF18"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="M11:N11"/>
-    <mergeCell ref="S11:V11"/>
-    <mergeCell ref="Y11:Z11"/>
-    <mergeCell ref="AC11:AF11"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="I10:J10"/>
-    <mergeCell ref="M10:N10"/>
-    <mergeCell ref="S10:V10"/>
-    <mergeCell ref="Y10:Z10"/>
-    <mergeCell ref="AC10:AF10"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="I6:J6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="S6:V6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AC6:AF6"/>
-    <mergeCell ref="R3:AF3"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="H5:J5"/>
-    <mergeCell ref="L5:N5"/>
-    <mergeCell ref="R5:V5"/>
-    <mergeCell ref="X5:Z5"/>
-    <mergeCell ref="AB5:AF5"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="I19:J19"/>
+    <mergeCell ref="M19:N19"/>
+    <mergeCell ref="S19:V19"/>
+    <mergeCell ref="Y19:Z19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="42" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF08279D-988E-4949-B1C3-65816486097A}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:Q15"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -2854,329 +2860,329 @@
   <sheetData>
     <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="76" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="116"/>
-      <c r="F2" s="108" t="s">
+      <c r="B2" s="77"/>
+      <c r="C2" s="78"/>
+      <c r="F2" s="79" t="s">
         <v>46</v>
       </c>
-      <c r="G2" s="109"/>
-      <c r="H2" s="109"/>
-      <c r="I2" s="109"/>
-      <c r="J2" s="109"/>
-      <c r="K2" s="109"/>
-      <c r="L2" s="109"/>
-      <c r="M2" s="109"/>
-      <c r="N2" s="109"/>
-      <c r="O2" s="109"/>
-      <c r="P2" s="109"/>
-      <c r="Q2" s="110"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="80"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="80"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="80"/>
+      <c r="Q2" s="81"/>
     </row>
     <row r="3" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="111" t="s">
+      <c r="A3" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="112">
+      <c r="B3" s="65">
         <v>1000</v>
       </c>
-      <c r="C3" s="113" t="s">
+      <c r="C3" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="100" t="s">
+      <c r="F3" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="93">
+      <c r="G3" s="49">
         <f>'Chemestry CH4'!B24</f>
         <v>50.010603792415168</v>
       </c>
-      <c r="H3" s="101" t="s">
+      <c r="H3" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="I3" s="117" t="s">
+      <c r="I3" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="118">
+      <c r="J3" s="68">
         <v>0</v>
       </c>
-      <c r="K3" s="119" t="s">
+      <c r="K3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="117" t="s">
+      <c r="L3" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="M3" s="118">
+      <c r="M3" s="68">
         <v>300</v>
       </c>
-      <c r="N3" s="119" t="s">
+      <c r="N3" s="69" t="s">
         <v>63</v>
       </c>
-      <c r="O3" s="117" t="s">
+      <c r="O3" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="P3" s="130">
+      <c r="P3" s="75">
         <v>21</v>
       </c>
-      <c r="Q3" s="119" t="s">
+      <c r="Q3" s="69" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F4" s="100" t="s">
+      <c r="F4" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="93">
+      <c r="G4" s="49">
         <f>G3*1000</f>
         <v>50010.603792415168</v>
       </c>
-      <c r="H4" s="101" t="s">
+      <c r="H4" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="102" t="s">
+      <c r="I4" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="103">
+      <c r="J4" s="59">
         <v>1013.25</v>
       </c>
-      <c r="K4" s="104" t="s">
+      <c r="K4" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="102" t="s">
+      <c r="L4" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="M4" s="103">
+      <c r="M4" s="59">
         <v>1</v>
       </c>
-      <c r="N4" s="104" t="s">
+      <c r="N4" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="O4" s="102" t="s">
+      <c r="O4" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="P4" s="103">
+      <c r="P4" s="59">
         <v>50</v>
       </c>
-      <c r="Q4" s="104" t="s">
+      <c r="Q4" s="60" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F5" s="102" t="s">
+      <c r="F5" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="103">
+      <c r="G5" s="59">
         <f>B3/G4</f>
         <v>1.9995759382366515E-2</v>
       </c>
-      <c r="H5" s="104" t="s">
+      <c r="H5" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="102" t="s">
+      <c r="I5" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="103">
+      <c r="J5" s="59">
         <f>J3+273.15</f>
         <v>273.14999999999998</v>
       </c>
-      <c r="K5" s="104" t="s">
+      <c r="K5" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="L5" s="102" t="s">
+      <c r="L5" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="M5" s="103">
+      <c r="M5" s="59">
         <f>M3</f>
         <v>300</v>
       </c>
-      <c r="N5" s="104" t="s">
+      <c r="N5" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="O5" s="102" t="s">
+      <c r="O5" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="P5" s="103">
+      <c r="P5" s="59">
         <f>P3/1000</f>
         <v>2.1000000000000001E-2</v>
       </c>
-      <c r="Q5" s="104" t="s">
+      <c r="Q5" s="60" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F6" s="102" t="s">
+      <c r="F6" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="128">
+      <c r="G6" s="74">
         <f>G5*'Chemestry CH4'!B29</f>
         <v>0.33964852763261294</v>
       </c>
-      <c r="H6" s="104" t="s">
+      <c r="H6" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="102" t="s">
+      <c r="I6" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="103">
+      <c r="J6" s="59">
         <f>J4*100</f>
         <v>101325</v>
       </c>
-      <c r="K6" s="104" t="s">
+      <c r="K6" s="60" t="s">
         <v>54</v>
       </c>
-      <c r="L6" s="102" t="s">
+      <c r="L6" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="M6" s="103">
+      <c r="M6" s="59">
         <f>M4*101325</f>
         <v>101325</v>
       </c>
-      <c r="N6" s="104" t="s">
+      <c r="N6" s="60" t="s">
         <v>54</v>
       </c>
-      <c r="O6" s="102" t="s">
+      <c r="O6" s="58" t="s">
         <v>62</v>
       </c>
-      <c r="P6" s="103">
+      <c r="P6" s="59">
         <f>P5*P4</f>
         <v>1.05</v>
       </c>
-      <c r="Q6" s="104" t="s">
+      <c r="Q6" s="60" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F7" s="102" t="s">
+      <c r="F7" s="58" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="128">
+      <c r="G7" s="74">
         <f>'Chemestry CH4'!B27</f>
         <v>5.8871915393654516E-2</v>
       </c>
-      <c r="H7" s="104" t="s">
+      <c r="H7" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="120" t="s">
+      <c r="I7" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="J7" s="129">
+      <c r="J7" s="74">
         <f>[1]!PropsSI("D", "T", J5, "P", J6, "Methane")</f>
         <v>0.71745877714291661</v>
       </c>
-      <c r="K7" s="121" t="s">
+      <c r="K7" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="L7" s="120" t="s">
+      <c r="L7" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="M7" s="129">
+      <c r="M7" s="74">
         <f>[1]!PropsSI("D", "T", M5, "P", M6, "Methane")</f>
         <v>0.65280527207610994</v>
       </c>
-      <c r="N7" s="121" t="s">
+      <c r="N7" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="O7" s="102" t="s">
+      <c r="O7" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="P7" s="103">
+      <c r="P7" s="59">
         <v>28.97</v>
       </c>
-      <c r="Q7" s="104" t="s">
+      <c r="Q7" s="60" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="F8" s="105" t="s">
+      <c r="F8" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="106">
+      <c r="G8" s="62">
         <v>8.3140000000000001</v>
       </c>
-      <c r="H8" s="107" t="s">
+      <c r="H8" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="I8" s="122" t="s">
+      <c r="I8" s="61" t="s">
         <v>66</v>
       </c>
-      <c r="J8" s="106">
+      <c r="J8" s="62">
         <f>[1]!PropsSI("D", "T", J5, "P", J6, "air")</f>
         <v>1.2930656163292633</v>
       </c>
-      <c r="K8" s="123" t="s">
+      <c r="K8" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="L8" s="122" t="s">
+      <c r="L8" s="61" t="s">
         <v>66</v>
       </c>
-      <c r="M8" s="106">
+      <c r="M8" s="62">
         <f>[1]!PropsSI("D", "T", M5, "P", M6, "air")</f>
         <v>1.1769955883877592</v>
       </c>
-      <c r="N8" s="123" t="s">
+      <c r="N8" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="O8" s="105" t="s">
+      <c r="O8" s="61" t="s">
         <v>83</v>
       </c>
       <c r="P8" s="20">
         <f>'Chemestry CH4'!C18</f>
         <v>16.032</v>
       </c>
-      <c r="Q8" s="104" t="s">
+      <c r="Q8" s="60" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="E10" s="99"/>
+      <c r="E10" s="55"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="1:17" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="124" t="s">
+      <c r="A12" s="70" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="125" t="s">
+      <c r="B12" s="71" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="125" t="s">
+      <c r="C12" s="71" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="125" t="s">
+      <c r="D12" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="125" t="s">
+      <c r="E12" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="125" t="s">
+      <c r="F12" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="G12" s="125" t="s">
+      <c r="G12" s="71" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="125" t="s">
+      <c r="H12" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="I12" s="127" t="s">
+      <c r="I12" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="127" t="s">
+      <c r="J12" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="K12" s="127" t="s">
+      <c r="K12" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="127" t="s">
+      <c r="L12" s="73" t="s">
         <v>77</v>
       </c>
-      <c r="M12" s="127" t="s">
+      <c r="M12" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="N12" s="125" t="s">
+      <c r="N12" s="71" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="126">
+      <c r="A13" s="72">
         <v>0.8</v>
       </c>
       <c r="B13" s="24" t="str">
@@ -3233,7 +3239,7 @@
       </c>
     </row>
     <row r="14" spans="1:17" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="126">
+      <c r="A14" s="72">
         <f>A13+0.2</f>
         <v>1</v>
       </c>
@@ -3291,7 +3297,7 @@
       </c>
     </row>
     <row r="15" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="126">
+      <c r="A15" s="72">
         <f>A14+0.2</f>
         <v>1.2</v>
       </c>
@@ -3312,7 +3318,7 @@
         <v>0.33964852763261294</v>
       </c>
       <c r="F15" s="24">
-        <f t="shared" ref="F14:F15" si="8">D15/($J$7*1000)*1000*60</f>
+        <f t="shared" ref="F15" si="8">D15/($J$7*1000)*1000*60</f>
         <v>2.0066583912508253</v>
       </c>
       <c r="G15" s="24">
@@ -3332,7 +3338,7 @@
         <v>0.88721804511278202</v>
       </c>
       <c r="K15" s="24">
-        <f t="shared" ref="K14:K15" si="9">I15*$P$8+J15*$P$7</f>
+        <f t="shared" ref="K15" si="9">I15*$P$8+J15*$P$7</f>
         <v>27.510827067669176</v>
       </c>
       <c r="L15" s="24">
@@ -3354,11 +3360,15 @@
     <mergeCell ref="F2:Q2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{308B74C1-373B-43F6-B438-35249E008B00}">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
@@ -3378,329 +3388,329 @@
   <sheetData>
     <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="114" t="s">
+      <c r="A2" s="76" t="s">
         <v>38</v>
       </c>
-      <c r="B2" s="115"/>
-      <c r="C2" s="116"/>
-      <c r="F2" s="108" t="s">
+      <c r="B2" s="77"/>
+      <c r="C2" s="78"/>
+      <c r="F2" s="79" t="s">
         <v>46</v>
       </c>
-      <c r="G2" s="109"/>
-      <c r="H2" s="109"/>
-      <c r="I2" s="109"/>
-      <c r="J2" s="109"/>
-      <c r="K2" s="109"/>
-      <c r="L2" s="109"/>
-      <c r="M2" s="109"/>
-      <c r="N2" s="109"/>
-      <c r="O2" s="109"/>
-      <c r="P2" s="109"/>
-      <c r="Q2" s="110"/>
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="80"/>
+      <c r="K2" s="80"/>
+      <c r="L2" s="80"/>
+      <c r="M2" s="80"/>
+      <c r="N2" s="80"/>
+      <c r="O2" s="80"/>
+      <c r="P2" s="80"/>
+      <c r="Q2" s="81"/>
     </row>
     <row r="3" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="111" t="s">
+      <c r="A3" s="64" t="s">
         <v>33</v>
       </c>
-      <c r="B3" s="112">
+      <c r="B3" s="65">
         <v>1000</v>
       </c>
-      <c r="C3" s="113" t="s">
+      <c r="C3" s="66" t="s">
         <v>34</v>
       </c>
-      <c r="F3" s="100" t="s">
+      <c r="F3" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="93">
-        <f>'Chemestry CH4'!B24</f>
-        <v>50.010603792415168</v>
-      </c>
-      <c r="H3" s="101" t="s">
+      <c r="G3" s="49">
+        <f>'Chemestry H2'!B24</f>
+        <v>119.94543650793651</v>
+      </c>
+      <c r="H3" s="57" t="s">
         <v>36</v>
       </c>
-      <c r="I3" s="117" t="s">
+      <c r="I3" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="J3" s="118">
+      <c r="J3" s="68">
         <v>0</v>
       </c>
-      <c r="K3" s="119" t="s">
+      <c r="K3" s="69" t="s">
         <v>13</v>
       </c>
-      <c r="L3" s="117" t="s">
+      <c r="L3" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="M3" s="118">
+      <c r="M3" s="68">
         <v>300</v>
       </c>
-      <c r="N3" s="119" t="s">
+      <c r="N3" s="69" t="s">
         <v>63</v>
       </c>
-      <c r="O3" s="117" t="s">
+      <c r="O3" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="P3" s="130">
+      <c r="P3" s="75">
         <v>4</v>
       </c>
-      <c r="Q3" s="119" t="s">
+      <c r="Q3" s="69" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F4" s="100" t="s">
+      <c r="F4" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="G4" s="93">
+      <c r="G4" s="49">
         <f>G3*1000</f>
-        <v>50010.603792415168</v>
-      </c>
-      <c r="H4" s="101" t="s">
+        <v>119945.43650793651</v>
+      </c>
+      <c r="H4" s="57" t="s">
         <v>37</v>
       </c>
-      <c r="I4" s="102" t="s">
+      <c r="I4" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="103">
+      <c r="J4" s="59">
         <v>1013.25</v>
       </c>
-      <c r="K4" s="104" t="s">
+      <c r="K4" s="60" t="s">
         <v>50</v>
       </c>
-      <c r="L4" s="102" t="s">
+      <c r="L4" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="M4" s="103">
+      <c r="M4" s="59">
         <v>1</v>
       </c>
-      <c r="N4" s="104" t="s">
+      <c r="N4" s="60" t="s">
         <v>64</v>
       </c>
-      <c r="O4" s="102" t="s">
+      <c r="O4" s="58" t="s">
         <v>58</v>
       </c>
-      <c r="P4" s="103">
+      <c r="P4" s="59">
         <v>50</v>
       </c>
-      <c r="Q4" s="104" t="s">
+      <c r="Q4" s="60" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F5" s="102" t="s">
+      <c r="F5" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="G5" s="103">
+      <c r="G5" s="59">
         <f>B3/G4</f>
-        <v>1.9995759382366515E-2</v>
-      </c>
-      <c r="H5" s="104" t="s">
+        <v>8.3371241884123894E-3</v>
+      </c>
+      <c r="H5" s="60" t="s">
         <v>40</v>
       </c>
-      <c r="I5" s="102" t="s">
+      <c r="I5" s="58" t="s">
         <v>51</v>
       </c>
-      <c r="J5" s="103">
+      <c r="J5" s="59">
         <f>J3+273.15</f>
         <v>273.14999999999998</v>
       </c>
-      <c r="K5" s="104" t="s">
+      <c r="K5" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="L5" s="102" t="s">
+      <c r="L5" s="58" t="s">
         <v>55</v>
       </c>
-      <c r="M5" s="103">
+      <c r="M5" s="59">
         <f>M3</f>
         <v>300</v>
       </c>
-      <c r="N5" s="104" t="s">
+      <c r="N5" s="60" t="s">
         <v>53</v>
       </c>
-      <c r="O5" s="102" t="s">
+      <c r="O5" s="58" t="s">
         <v>60</v>
       </c>
-      <c r="P5" s="103">
+      <c r="P5" s="59">
         <f>P3/1000</f>
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="Q5" s="104" t="s">
+      <c r="Q5" s="60" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F6" s="102" t="s">
+      <c r="F6" s="58" t="s">
         <v>41</v>
       </c>
-      <c r="G6" s="128">
+      <c r="G6" s="74">
         <f>G5*'Chemestry H2'!B29</f>
-        <v>0.67525362041245673</v>
-      </c>
-      <c r="H6" s="104" t="s">
+        <v>0.28154336048964068</v>
+      </c>
+      <c r="H6" s="60" t="s">
         <v>42</v>
       </c>
-      <c r="I6" s="102" t="s">
+      <c r="I6" s="58" t="s">
         <v>52</v>
       </c>
-      <c r="J6" s="103">
+      <c r="J6" s="59">
         <f>J4*100</f>
         <v>101325</v>
       </c>
-      <c r="K6" s="104" t="s">
+      <c r="K6" s="60" t="s">
         <v>54</v>
       </c>
-      <c r="L6" s="102" t="s">
+      <c r="L6" s="58" t="s">
         <v>56</v>
       </c>
-      <c r="M6" s="103">
+      <c r="M6" s="59">
         <f>M4*101325</f>
         <v>101325</v>
       </c>
-      <c r="N6" s="104" t="s">
+      <c r="N6" s="60" t="s">
         <v>54</v>
       </c>
-      <c r="O6" s="102" t="s">
+      <c r="O6" s="58" t="s">
         <v>62</v>
       </c>
-      <c r="P6" s="103">
+      <c r="P6" s="59">
         <f>P5*P4</f>
         <v>0.2</v>
       </c>
-      <c r="Q6" s="104" t="s">
+      <c r="Q6" s="60" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="F7" s="102" t="s">
+      <c r="F7" s="58" t="s">
         <v>71</v>
       </c>
-      <c r="G7" s="128">
+      <c r="G7" s="74">
         <f>'Chemestry H2'!B27</f>
         <v>2.9612220916568736E-2</v>
       </c>
-      <c r="H7" s="104" t="s">
+      <c r="H7" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="I7" s="120" t="s">
+      <c r="I7" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="J7" s="129">
+      <c r="J7" s="74">
         <f>[1]!PropsSI("D", "T", J5, "P", J6, "H2")</f>
         <v>8.9882376384805382E-2</v>
       </c>
-      <c r="K7" s="121" t="s">
+      <c r="K7" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="L7" s="120" t="s">
+      <c r="L7" s="58" t="s">
         <v>65</v>
       </c>
-      <c r="M7" s="129">
+      <c r="M7" s="74">
         <f>[1]!PropsSI("D", "T", M5, "P", M6, "H2")</f>
         <v>8.1840487796729228E-2</v>
       </c>
-      <c r="N7" s="121" t="s">
+      <c r="N7" s="60" t="s">
         <v>67</v>
       </c>
-      <c r="O7" s="102" t="s">
+      <c r="O7" s="58" t="s">
         <v>73</v>
       </c>
-      <c r="P7" s="103">
+      <c r="P7" s="59">
         <v>28.97</v>
       </c>
-      <c r="Q7" s="104" t="s">
+      <c r="Q7" s="60" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="F8" s="105" t="s">
+      <c r="F8" s="61" t="s">
         <v>75</v>
       </c>
-      <c r="G8" s="106">
+      <c r="G8" s="62">
         <v>8.3140000000000001</v>
       </c>
-      <c r="H8" s="107" t="s">
+      <c r="H8" s="63" t="s">
         <v>76</v>
       </c>
-      <c r="I8" s="122" t="s">
+      <c r="I8" s="61" t="s">
         <v>66</v>
       </c>
-      <c r="J8" s="106">
+      <c r="J8" s="62">
         <f>[1]!PropsSI("D", "T", J5, "P", J6, "air")</f>
         <v>1.2930656163292633</v>
       </c>
-      <c r="K8" s="123" t="s">
+      <c r="K8" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="L8" s="122" t="s">
+      <c r="L8" s="61" t="s">
         <v>66</v>
       </c>
-      <c r="M8" s="106">
+      <c r="M8" s="62">
         <f>[1]!PropsSI("D", "T", M5, "P", M6, "air")</f>
         <v>1.1769955883877592</v>
       </c>
-      <c r="N8" s="123" t="s">
+      <c r="N8" s="63" t="s">
         <v>67</v>
       </c>
-      <c r="O8" s="105" t="s">
+      <c r="O8" s="61" t="s">
         <v>83</v>
       </c>
       <c r="P8" s="20">
         <f>'Chemestry H2'!C18</f>
         <v>2.016</v>
       </c>
-      <c r="Q8" s="104" t="s">
+      <c r="Q8" s="60" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="E10" s="99"/>
+      <c r="E10" s="55"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="12" spans="1:17" ht="45.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="124" t="s">
+      <c r="A12" s="70" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="125" t="s">
+      <c r="B12" s="71" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="125" t="s">
+      <c r="C12" s="71" t="s">
         <v>45</v>
       </c>
-      <c r="D12" s="125" t="s">
+      <c r="D12" s="71" t="s">
         <v>49</v>
       </c>
-      <c r="E12" s="125" t="s">
+      <c r="E12" s="71" t="s">
         <v>48</v>
       </c>
-      <c r="F12" s="125" t="s">
+      <c r="F12" s="71" t="s">
         <v>68</v>
       </c>
-      <c r="G12" s="125" t="s">
+      <c r="G12" s="71" t="s">
         <v>69</v>
       </c>
-      <c r="H12" s="125" t="s">
+      <c r="H12" s="71" t="s">
         <v>70</v>
       </c>
-      <c r="I12" s="127" t="s">
+      <c r="I12" s="73" t="s">
         <v>80</v>
       </c>
-      <c r="J12" s="127" t="s">
+      <c r="J12" s="73" t="s">
         <v>81</v>
       </c>
-      <c r="K12" s="127" t="s">
+      <c r="K12" s="73" t="s">
         <v>82</v>
       </c>
-      <c r="L12" s="127" t="s">
+      <c r="L12" s="73" t="s">
         <v>77</v>
       </c>
-      <c r="M12" s="127" t="s">
+      <c r="M12" s="73" t="s">
         <v>78</v>
       </c>
-      <c r="N12" s="125" t="s">
+      <c r="N12" s="71" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="126">
+      <c r="A13" s="72">
         <v>0.5</v>
       </c>
       <c r="B13" s="24" t="str">
@@ -3713,19 +3723,19 @@
       </c>
       <c r="D13" s="24">
         <f>IF($A13=1,$G$5,IF($A13&gt;1,E13*C13,$G$5))</f>
-        <v>1.9995759382366515E-2</v>
+        <v>8.3371241884123894E-3</v>
       </c>
       <c r="E13" s="24">
         <f>IF($A13=1,$G$6,IF($A13&gt;1,$G$6,D13/C13))</f>
-        <v>1.3505072408249135</v>
+        <v>0.56308672097928136</v>
       </c>
       <c r="F13" s="24">
         <f>D13/($J$7*1000)*1000*60</f>
-        <v>13.347951080038511</v>
+        <v>5.5653563181636887</v>
       </c>
       <c r="G13" s="24">
         <f>E13/($J$8*1000)*1000*60</f>
-        <v>62.665369356524131</v>
+        <v>26.12798827229344</v>
       </c>
       <c r="H13" s="24">
         <f>IF(A13&gt;1,E13*$G$7*$G$4,D13*$G$4)</f>
@@ -3749,44 +3759,44 @@
       </c>
       <c r="M13" s="24">
         <f>(D13+E13)/(1000*L13*PI()*($P$5/2)^2)</f>
-        <v>97.219385952421874</v>
+        <v>40.535099403192014</v>
       </c>
       <c r="N13" s="24">
         <f>M13*L13*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>23533.292372663094</v>
+        <v>9812.079517526674</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="126">
+      <c r="A14" s="72">
         <f>A13+0.1</f>
         <v>0.6</v>
       </c>
       <c r="B14" s="24" t="str">
-        <f t="shared" ref="B14:B31" si="0">IF($A14=1,"Stoc",IF($A14&gt;1,"air","Fuel"))</f>
+        <f t="shared" ref="B14:B21" si="0">IF($A14=1,"Stoc",IF($A14&gt;1,"air","Fuel"))</f>
         <v>Fuel</v>
       </c>
       <c r="C14" s="24">
-        <f t="shared" ref="C14:C15" si="1">A14*$G$7</f>
+        <f t="shared" ref="C14" si="1">A14*$G$7</f>
         <v>1.7767332549941242E-2</v>
       </c>
       <c r="D14" s="24">
-        <f t="shared" ref="D14:D31" si="2">IF($A14=1,$G$5,IF($A14&gt;1,E14*C14,$G$5))</f>
-        <v>1.9995759382366515E-2</v>
+        <f t="shared" ref="D14:D21" si="2">IF($A14=1,$G$5,IF($A14&gt;1,E14*C14,$G$5))</f>
+        <v>8.3371241884123894E-3</v>
       </c>
       <c r="E14" s="24">
-        <f t="shared" ref="E14:E15" si="3">IF($A14=1,$G$6,IF($A14&gt;1,$G$6,D14/C14))</f>
-        <v>1.1254227006874278</v>
+        <f t="shared" ref="E14" si="3">IF($A14=1,$G$6,IF($A14&gt;1,$G$6,D14/C14))</f>
+        <v>0.4692389341494011</v>
       </c>
       <c r="F14" s="24">
-        <f t="shared" ref="F14:F15" si="4">D14/($J$7*1000)*1000*60</f>
-        <v>13.347951080038511</v>
+        <f t="shared" ref="F14" si="4">D14/($J$7*1000)*1000*60</f>
+        <v>5.5653563181636887</v>
       </c>
       <c r="G14" s="24">
-        <f t="shared" ref="G14:G15" si="5">E14/($J$8*1000)*1000*60</f>
-        <v>52.22114113043677</v>
+        <f t="shared" ref="G14" si="5">E14/($J$8*1000)*1000*60</f>
+        <v>21.773323560244535</v>
       </c>
       <c r="H14" s="24">
-        <f t="shared" ref="H14:H15" si="6">IF(A14&gt;1,E14*$G$7*$G$4,D14*$G$4)</f>
+        <f t="shared" ref="H14" si="6">IF(A14&gt;1,E14*$G$7*$G$4,D14*$G$4)</f>
         <v>1000</v>
       </c>
       <c r="I14" s="24">
@@ -3794,7 +3804,7 @@
         <v>5.97609561752988E-2</v>
       </c>
       <c r="J14" s="24">
-        <f t="shared" ref="J14:J31" si="7">1-I14</f>
+        <f t="shared" ref="J14:J21" si="7">1-I14</f>
         <v>0.94023904382470125</v>
       </c>
       <c r="K14" s="24">
@@ -3802,20 +3812,20 @@
         <v>27.359203187250998</v>
       </c>
       <c r="L14" s="24">
-        <f t="shared" ref="L14:L31" si="8">($M$6*K14)/($G$8*$M$5) /1000</f>
+        <f t="shared" ref="L14:L21" si="8">($M$6*K14)/($G$8*$M$5) /1000</f>
         <v>1.1114470623639674</v>
       </c>
       <c r="M14" s="24">
         <f>(D14+E14)/(1000*L14*PI()*($P$5/2)^2)</f>
-        <v>82.009758270032989</v>
+        <v>34.193527051635563</v>
       </c>
       <c r="N14" s="24">
         <f>M14*L14*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>19668.302445008256</v>
+        <v>8200.5927818822365</v>
       </c>
     </row>
     <row r="15" spans="1:17" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="126">
+      <c r="A15" s="72">
         <f>A14+0.1</f>
         <v>0.7</v>
       </c>
@@ -3824,27 +3834,27 @@
         <v>Fuel</v>
       </c>
       <c r="C15" s="24">
-        <f t="shared" ref="C15:C16" si="9">A15*$G$7</f>
+        <f t="shared" ref="C15" si="9">A15*$G$7</f>
         <v>2.0728554641598115E-2</v>
       </c>
       <c r="D15" s="24">
         <f t="shared" si="2"/>
-        <v>1.9995759382366515E-2</v>
+        <v>8.3371241884123894E-3</v>
       </c>
       <c r="E15" s="24">
-        <f t="shared" ref="E15:E16" si="10">IF($A15=1,$G$6,IF($A15&gt;1,$G$6,D15/C15))</f>
-        <v>0.9646480291606524</v>
+        <f t="shared" ref="E15" si="10">IF($A15=1,$G$6,IF($A15&gt;1,$G$6,D15/C15))</f>
+        <v>0.40220480069948666</v>
       </c>
       <c r="F15" s="24">
-        <f t="shared" ref="F15:F16" si="11">D15/($J$7*1000)*1000*60</f>
-        <v>13.347951080038511</v>
+        <f t="shared" ref="F15" si="11">D15/($J$7*1000)*1000*60</f>
+        <v>5.5653563181636887</v>
       </c>
       <c r="G15" s="24">
-        <f t="shared" ref="G15:G16" si="12">E15/($J$8*1000)*1000*60</f>
-        <v>44.760978111802942</v>
+        <f t="shared" ref="G15" si="12">E15/($J$8*1000)*1000*60</f>
+        <v>18.662848765923883</v>
       </c>
       <c r="H15" s="24">
-        <f t="shared" ref="H15:H16" si="13">IF(A15&gt;1,E15*$G$7*$G$4,D15*$G$4)</f>
+        <f t="shared" ref="H15" si="13">IF(A15&gt;1,E15*$G$7*$G$4,D15*$G$4)</f>
         <v>1000</v>
       </c>
       <c r="I15" s="24">
@@ -3865,15 +3875,15 @@
       </c>
       <c r="M15" s="24">
         <f>(D15+E15)/(1000*L15*PI()*($P$5/2)^2)</f>
-        <v>71.14856046635424</v>
+        <v>29.665009119776705</v>
       </c>
       <c r="N15" s="24">
         <f>M15*L15*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>16907.595353826233</v>
+        <v>7049.530827850499</v>
       </c>
     </row>
     <row r="16" spans="1:17" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="126">
+      <c r="A16" s="72">
         <f t="shared" ref="A16:A21" si="14">A15+0.1</f>
         <v>0.79999999999999993</v>
       </c>
@@ -3887,19 +3897,19 @@
       </c>
       <c r="D16" s="24">
         <f t="shared" si="2"/>
-        <v>1.9995759382366515E-2</v>
+        <v>8.3371241884123894E-3</v>
       </c>
       <c r="E16" s="24">
         <f t="shared" ref="E16:E21" si="16">IF($A16=1,$G$6,IF($A16&gt;1,$G$6,D16/C16))</f>
-        <v>0.84406702551557089</v>
+        <v>0.35192920061205085</v>
       </c>
       <c r="F16" s="24">
         <f t="shared" ref="F16:F21" si="17">D16/($J$7*1000)*1000*60</f>
-        <v>13.347951080038511</v>
+        <v>5.5653563181636887</v>
       </c>
       <c r="G16" s="24">
         <f t="shared" ref="G16:G21" si="18">E16/($J$8*1000)*1000*60</f>
-        <v>39.165855847827586</v>
+        <v>16.329992670183405</v>
       </c>
       <c r="H16" s="24">
         <f t="shared" ref="H16:H21" si="19">IF(A16&gt;1,E16*$G$7*$G$4,D16*$G$4)</f>
@@ -3923,15 +3933,15 @@
       </c>
       <c r="M16" s="24">
         <f t="shared" ref="M16:M21" si="21">(D16+E16)/(1000*L16*PI()*($P$5/2)^2)</f>
-        <v>63.005125908142681</v>
+        <v>26.269647936750523</v>
       </c>
       <c r="N16" s="24">
         <f>M16*L16*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>14837.065035439715</v>
+        <v>6186.2343623266961</v>
       </c>
     </row>
     <row r="17" spans="1:14" ht="25.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="126">
+      <c r="A17" s="72">
         <f t="shared" si="14"/>
         <v>0.89999999999999991</v>
       </c>
@@ -3945,19 +3955,19 @@
       </c>
       <c r="D17" s="24">
         <f t="shared" si="2"/>
-        <v>1.9995759382366515E-2</v>
+        <v>8.3371241884123894E-3</v>
       </c>
       <c r="E17" s="24">
         <f t="shared" si="16"/>
-        <v>0.7502818004582853</v>
+        <v>0.31282595609960079</v>
       </c>
       <c r="F17" s="24">
         <f t="shared" si="17"/>
-        <v>13.347951080038511</v>
+        <v>5.5653563181636887</v>
       </c>
       <c r="G17" s="24">
         <f t="shared" si="18"/>
-        <v>34.814094086957851</v>
+        <v>14.515549040163023</v>
       </c>
       <c r="H17" s="24">
         <f t="shared" si="19"/>
@@ -3981,15 +3991,15 @@
       </c>
       <c r="M17" s="24">
         <f t="shared" si="21"/>
-        <v>56.673528702176384</v>
+        <v>23.629722580192322</v>
       </c>
       <c r="N17" s="24">
         <f>M17*L17*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>13226.652565583536</v>
+        <v>5514.7815558081829</v>
       </c>
     </row>
     <row r="18" spans="1:14" ht="24.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="126">
+      <c r="A18" s="72">
         <f t="shared" si="14"/>
         <v>0.99999999999999989</v>
       </c>
@@ -4003,19 +4013,19 @@
       </c>
       <c r="D18" s="24">
         <f t="shared" si="2"/>
-        <v>1.9995759382366515E-2</v>
+        <v>8.3371241884123894E-3</v>
       </c>
       <c r="E18" s="24">
         <f t="shared" si="16"/>
-        <v>0.67525362041245673</v>
+        <v>0.28154336048964068</v>
       </c>
       <c r="F18" s="24">
         <f t="shared" si="17"/>
-        <v>13.347951080038511</v>
+        <v>5.5653563181636887</v>
       </c>
       <c r="G18" s="24">
         <f t="shared" si="18"/>
-        <v>31.332684678262066</v>
+        <v>13.06399413614672</v>
       </c>
       <c r="H18" s="24">
         <f t="shared" si="19"/>
@@ -4039,15 +4049,15 @@
       </c>
       <c r="M18" s="24">
         <f t="shared" si="21"/>
-        <v>51.610213325197371</v>
+        <v>21.518600501968145</v>
       </c>
       <c r="N18" s="24">
         <f>M18*L18*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>11938.32258969859</v>
+        <v>4977.6193105933708</v>
       </c>
     </row>
     <row r="19" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="126">
+      <c r="A19" s="72">
         <f t="shared" si="14"/>
         <v>1.0999999999999999</v>
       </c>
@@ -4061,19 +4071,19 @@
       </c>
       <c r="D19" s="24">
         <f t="shared" si="2"/>
-        <v>2.1995335320603167E-2</v>
+        <v>9.1708366072536275E-3</v>
       </c>
       <c r="E19" s="24">
         <f t="shared" si="16"/>
-        <v>0.67525362041245673</v>
+        <v>0.28154336048964068</v>
       </c>
       <c r="F19" s="24">
         <f t="shared" si="17"/>
-        <v>14.68274618804236</v>
+        <v>6.1218919499800561</v>
       </c>
       <c r="G19" s="24">
         <f t="shared" si="18"/>
-        <v>31.332684678262066</v>
+        <v>13.06399413614672</v>
       </c>
       <c r="H19" s="24">
         <f t="shared" si="19"/>
@@ -4097,15 +4107,15 @@
       </c>
       <c r="M19" s="24">
         <f t="shared" si="21"/>
-        <v>52.216208901274491</v>
+        <v>21.771267093857571</v>
       </c>
       <c r="N19" s="24">
         <f>M19*L19*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>11972.657870371993</v>
+        <v>4991.9352209593771</v>
       </c>
     </row>
     <row r="20" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="126">
+      <c r="A20" s="72">
         <f t="shared" si="14"/>
         <v>1.2</v>
       </c>
@@ -4119,19 +4129,19 @@
       </c>
       <c r="D20" s="24">
         <f t="shared" si="2"/>
-        <v>2.3994911258839822E-2</v>
+        <v>1.0004549026094867E-2</v>
       </c>
       <c r="E20" s="24">
         <f t="shared" si="16"/>
-        <v>0.67525362041245673</v>
+        <v>0.28154336048964068</v>
       </c>
       <c r="F20" s="24">
         <f t="shared" si="17"/>
-        <v>16.017541296046218</v>
+        <v>6.6784275817964271</v>
       </c>
       <c r="G20" s="24">
         <f t="shared" si="18"/>
-        <v>31.332684678262066</v>
+        <v>13.06399413614672</v>
       </c>
       <c r="H20" s="24">
         <f t="shared" si="19"/>
@@ -4155,15 +4165,15 @@
       </c>
       <c r="M20" s="24">
         <f t="shared" si="21"/>
-        <v>52.824158267817261</v>
+        <v>22.024748308159612</v>
       </c>
       <c r="N20" s="24">
         <f>M20*L20*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>12006.993151045408</v>
+        <v>5006.2511313253854</v>
       </c>
     </row>
     <row r="21" spans="1:14" ht="25.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="126">
+      <c r="A21" s="72">
         <f t="shared" si="14"/>
         <v>1.3</v>
       </c>
@@ -4177,19 +4187,19 @@
       </c>
       <c r="D21" s="24">
         <f t="shared" si="2"/>
-        <v>2.5994487197076473E-2</v>
+        <v>1.0838261444936107E-2</v>
       </c>
       <c r="E21" s="24">
         <f t="shared" si="16"/>
-        <v>0.67525362041245673</v>
+        <v>0.28154336048964068</v>
       </c>
       <c r="F21" s="24">
         <f t="shared" si="17"/>
-        <v>17.352336404050064</v>
+        <v>7.2349632136127964</v>
       </c>
       <c r="G21" s="24">
         <f t="shared" si="18"/>
-        <v>31.332684678262066</v>
+        <v>13.06399413614672</v>
       </c>
       <c r="H21" s="24">
         <f t="shared" si="19"/>
@@ -4213,11 +4223,11 @@
       </c>
       <c r="M21" s="24">
         <f t="shared" si="21"/>
-        <v>53.434057144989545</v>
+        <v>22.279042360419648</v>
       </c>
       <c r="N21" s="24">
         <f>M21*L21*$P$5/([1]!PropsSI("V","T",$M$5,"P",$M$6,"Air"))</f>
-        <v>12041.328431718814</v>
+        <v>5020.5670416913908</v>
       </c>
     </row>
   </sheetData>
@@ -4226,5 +4236,6 @@
     <mergeCell ref="F2:Q2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="60" fitToHeight="0" orientation="landscape" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>